<commit_message>
Hub View Improved. Product Lef. Overall Page left.
</commit_message>
<xml_diff>
--- a/outputs/route_analysis.xlsx
+++ b/outputs/route_analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="57">
   <si>
     <t>Source</t>
   </si>
@@ -28,166 +28,163 @@
     <t>Products</t>
   </si>
   <si>
-    <t>189, 1167, 1296, 4145, 7310, 8529, 13490, 14248, 14654, 15300, 16407, 18098, 19690, 20308, 23081, 23638</t>
-  </si>
-  <si>
-    <t>2122, 7310, 8529, 18098, 23081</t>
-  </si>
-  <si>
-    <t>189, 14654, 16336</t>
-  </si>
-  <si>
-    <t>189, 6151, 18098, 20661, 23638</t>
-  </si>
-  <si>
-    <t>189, 14248, 16407, 20827, 23638, 25885</t>
-  </si>
-  <si>
-    <t>189, 2122, 4145, 6982, 14248, 14788, 15300, 16984</t>
-  </si>
-  <si>
-    <t>189, 1167, 14248, 23638</t>
-  </si>
-  <si>
-    <t>13179, 16336</t>
-  </si>
-  <si>
-    <t>6151, 13179, 16336, 25598</t>
-  </si>
-  <si>
-    <t>14654, 16336</t>
-  </si>
-  <si>
-    <t>189, 16336, 25598</t>
-  </si>
-  <si>
-    <t>13179, 20661</t>
-  </si>
-  <si>
-    <t>6151, 13179, 16336</t>
+    <t>2122, 7310, 8529, 13179, 14654, 23081, 25570</t>
+  </si>
+  <si>
+    <t>16336, 23401, 23638</t>
+  </si>
+  <si>
+    <t>1296, 2122, 4145, 6151, 6982, 7310, 13490, 14248, 15300, 16407, 19690, 23081</t>
+  </si>
+  <si>
+    <t>16336, 23638</t>
   </si>
   <si>
     <t>16336</t>
   </si>
   <si>
-    <t>13179, 16336, 20661</t>
+    <t>1167, 6151, 13179, 14654, 19690</t>
+  </si>
+  <si>
+    <t>1167, 6151</t>
+  </si>
+  <si>
+    <t>189, 6151, 20661</t>
+  </si>
+  <si>
+    <t>13179</t>
+  </si>
+  <si>
+    <t>1296, 6982, 16336, 25598</t>
+  </si>
+  <si>
+    <t>189, 1167</t>
+  </si>
+  <si>
+    <t>13179, 20827, 23401, 25885</t>
+  </si>
+  <si>
+    <t>1167, 6151, 6982, 14654, 20827, 23401, 25885</t>
+  </si>
+  <si>
+    <t>23081, 23638</t>
+  </si>
+  <si>
+    <t>6151, 23081</t>
+  </si>
+  <si>
+    <t>13179, 14654</t>
+  </si>
+  <si>
+    <t>14248, 14788, 23638</t>
+  </si>
+  <si>
+    <t>1296, 6151, 16984</t>
+  </si>
+  <si>
+    <t>1167, 6982, 8529, 23401, 25885</t>
+  </si>
+  <si>
+    <t>1296, 6151, 6982, 14248, 23401, 24768</t>
+  </si>
+  <si>
+    <t>2122, 6982, 14788, 15300, 16984, 25885</t>
+  </si>
+  <si>
+    <t>7310</t>
+  </si>
+  <si>
+    <t>189, 14788, 23638</t>
+  </si>
+  <si>
+    <t>19690, 23081, 23638</t>
+  </si>
+  <si>
+    <t>1167, 6151, 14654</t>
+  </si>
+  <si>
+    <t>14788, 20661</t>
+  </si>
+  <si>
+    <t>2122, 14654, 15305, 16407</t>
+  </si>
+  <si>
+    <t>14788, 23638, 25598</t>
+  </si>
+  <si>
+    <t>1167, 19690</t>
+  </si>
+  <si>
+    <t>5159, 14654, 14788</t>
+  </si>
+  <si>
+    <t>23638</t>
   </si>
   <si>
     <t>189</t>
   </si>
   <si>
-    <t>13179</t>
-  </si>
-  <si>
-    <t>6151, 18098</t>
+    <t>20661</t>
   </si>
   <si>
     <t>6151</t>
   </si>
   <si>
-    <t>2122, 6151, 14788, 23081, 23638</t>
-  </si>
-  <si>
-    <t>6151, 23401</t>
-  </si>
-  <si>
-    <t>8529, 14654, 18098, 19690</t>
+    <t>14788, 23638</t>
+  </si>
+  <si>
+    <t>6982, 13490, 14248, 15300, 15305, 16998, 23401</t>
+  </si>
+  <si>
+    <t>1167, 14654</t>
+  </si>
+  <si>
+    <t>14654</t>
+  </si>
+  <si>
+    <t>1167, 25598</t>
+  </si>
+  <si>
+    <t>5159, 13678, 15300</t>
+  </si>
+  <si>
+    <t>6982</t>
+  </si>
+  <si>
+    <t>23401, 23638</t>
+  </si>
+  <si>
+    <t>14788</t>
+  </si>
+  <si>
+    <t>1167</t>
+  </si>
+  <si>
+    <t>14248</t>
+  </si>
+  <si>
+    <t>1296</t>
+  </si>
+  <si>
+    <t>14654, 23081</t>
+  </si>
+  <si>
+    <t>25598</t>
+  </si>
+  <si>
+    <t>23081</t>
+  </si>
+  <si>
+    <t>16407, 16984, 19690</t>
+  </si>
+  <si>
+    <t>20661, 23081</t>
   </si>
   <si>
     <t>6151, 14654</t>
   </si>
   <si>
-    <t>4145, 14248, 16407, 23081, 23401, 23638, 24768</t>
-  </si>
-  <si>
-    <t>14788, 25570</t>
-  </si>
-  <si>
-    <t>1296, 7310</t>
-  </si>
-  <si>
-    <t>14788</t>
-  </si>
-  <si>
-    <t>14248, 14788, 23638</t>
-  </si>
-  <si>
-    <t>23401, 23638</t>
-  </si>
-  <si>
-    <t>189, 14248</t>
-  </si>
-  <si>
-    <t>14654, 23401, 23638</t>
-  </si>
-  <si>
-    <t>5159, 6151, 20661, 23081</t>
-  </si>
-  <si>
-    <t>13179, 14654</t>
-  </si>
-  <si>
-    <t>23401, 25598</t>
-  </si>
-  <si>
-    <t>18098</t>
-  </si>
-  <si>
-    <t>1296, 6982, 13490, 14248, 16998</t>
-  </si>
-  <si>
-    <t>20661, 23401, 23638</t>
-  </si>
-  <si>
-    <t>14654</t>
-  </si>
-  <si>
-    <t>23401</t>
-  </si>
-  <si>
-    <t>15300, 19690, 23081</t>
-  </si>
-  <si>
-    <t>6151, 19690, 25885</t>
-  </si>
-  <si>
-    <t>20661, 25598</t>
-  </si>
-  <si>
-    <t>23401, 25885</t>
-  </si>
-  <si>
-    <t>6982, 14248, 23401</t>
-  </si>
-  <si>
-    <t>25885</t>
-  </si>
-  <si>
-    <t>8529, 16407, 16984</t>
-  </si>
-  <si>
-    <t>20661</t>
-  </si>
-  <si>
-    <t>13678, 15300</t>
-  </si>
-  <si>
-    <t>15300</t>
-  </si>
-  <si>
-    <t>25598</t>
-  </si>
-  <si>
-    <t>6151, 20661</t>
-  </si>
-  <si>
-    <t>5159, 23081</t>
-  </si>
-  <si>
-    <t>5159</t>
-  </si>
-  <si>
-    <t>15300, 25885</t>
+    <t>1296, 23081</t>
   </si>
 </sst>
 </file>
@@ -545,7 +542,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D85"/>
+  <dimension ref="A1:D88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -564,13 +561,13 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2">
-        <v>4108</v>
+        <v>4301</v>
       </c>
       <c r="B2">
-        <v>4101</v>
+        <v>4304</v>
       </c>
       <c r="C2">
-        <v>46913.74</v>
+        <v>52009.68</v>
       </c>
       <c r="D2" t="s">
         <v>4</v>
@@ -578,13 +575,13 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3">
+        <v>4108</v>
+      </c>
+      <c r="B3">
         <v>4301</v>
       </c>
-      <c r="B3">
-        <v>4304</v>
-      </c>
       <c r="C3">
-        <v>23913.79</v>
+        <v>24630.14</v>
       </c>
       <c r="D3" t="s">
         <v>5</v>
@@ -592,13 +589,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4">
-        <v>2000</v>
+        <v>4108</v>
       </c>
       <c r="B4">
-        <v>4301</v>
+        <v>4101</v>
       </c>
       <c r="C4">
-        <v>21299.86</v>
+        <v>24193.29</v>
       </c>
       <c r="D4" t="s">
         <v>6</v>
@@ -606,13 +603,13 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5">
-        <v>4400</v>
+        <v>4403</v>
       </c>
       <c r="B5">
-        <v>4401</v>
+        <v>4101</v>
       </c>
       <c r="C5">
-        <v>19952.47</v>
+        <v>19356.09</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
@@ -623,251 +620,251 @@
         <v>4108</v>
       </c>
       <c r="B6">
-        <v>4401</v>
+        <v>4304</v>
       </c>
       <c r="C6">
-        <v>18368.01</v>
+        <v>16047.2</v>
       </c>
       <c r="D6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7">
-        <v>4108</v>
+        <v>4200</v>
       </c>
       <c r="B7">
-        <v>4200</v>
+        <v>4203</v>
       </c>
       <c r="C7">
-        <v>18072.1</v>
+        <v>14847.5</v>
       </c>
       <c r="D7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8">
-        <v>4108</v>
+        <v>4105</v>
       </c>
       <c r="B8">
         <v>4403</v>
       </c>
       <c r="C8">
-        <v>17708.89</v>
+        <v>11008.18</v>
       </c>
       <c r="D8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9">
-        <v>4100</v>
+        <v>4105</v>
       </c>
       <c r="B9">
-        <v>4301</v>
+        <v>4304</v>
       </c>
       <c r="C9">
-        <v>13217.87</v>
+        <v>10471.89</v>
       </c>
       <c r="D9" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10">
-        <v>4104</v>
+        <v>4400</v>
       </c>
       <c r="B10">
-        <v>4301</v>
+        <v>4401</v>
       </c>
       <c r="C10">
-        <v>12243.39</v>
+        <v>9907.34</v>
       </c>
       <c r="D10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11">
+        <v>4400</v>
+      </c>
+      <c r="B11">
         <v>4404</v>
       </c>
-      <c r="B11">
-        <v>4101</v>
-      </c>
       <c r="C11">
-        <v>12034.61</v>
+        <v>8234.74</v>
       </c>
       <c r="D11" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12">
-        <v>4201</v>
+        <v>4100</v>
       </c>
       <c r="B12">
-        <v>4200</v>
+        <v>4403</v>
       </c>
       <c r="C12">
-        <v>10339.79</v>
+        <v>8096.46</v>
       </c>
       <c r="D12" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13">
-        <v>4302</v>
+        <v>4104</v>
       </c>
       <c r="B13">
         <v>4301</v>
       </c>
       <c r="C13">
-        <v>8873.16</v>
+        <v>7996.259999999999</v>
       </c>
       <c r="D13" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14">
-        <v>4105</v>
+        <v>4201</v>
       </c>
       <c r="B14">
-        <v>4304</v>
+        <v>4403</v>
       </c>
       <c r="C14">
-        <v>7900.249999999999</v>
+        <v>7804.09</v>
       </c>
       <c r="D14" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15">
-        <v>4105</v>
+        <v>4108</v>
       </c>
       <c r="B15">
-        <v>4203</v>
+        <v>4403</v>
       </c>
       <c r="C15">
-        <v>6703.02</v>
+        <v>7370.35</v>
       </c>
       <c r="D15" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16">
-        <v>4302</v>
+        <v>4108</v>
       </c>
       <c r="B16">
-        <v>4304</v>
+        <v>4401</v>
       </c>
       <c r="C16">
-        <v>6230.87</v>
+        <v>7103.71</v>
       </c>
       <c r="D16" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17">
-        <v>2000</v>
+        <v>4401</v>
       </c>
       <c r="B17">
-        <v>4203</v>
+        <v>4101</v>
       </c>
       <c r="C17">
-        <v>6216.41</v>
+        <v>6678.08</v>
       </c>
       <c r="D17" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18">
-        <v>4108</v>
+        <v>4203</v>
       </c>
       <c r="B18">
-        <v>4301</v>
+        <v>4302</v>
       </c>
       <c r="C18">
-        <v>6041.6</v>
+        <v>6180.85</v>
       </c>
       <c r="D18" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19">
-        <v>4105</v>
+        <v>4100</v>
       </c>
       <c r="B19">
-        <v>4401</v>
+        <v>4301</v>
       </c>
       <c r="C19">
-        <v>5462.67</v>
+        <v>5986.88</v>
       </c>
       <c r="D19" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20">
-        <v>4104</v>
+        <v>4101</v>
       </c>
       <c r="B20">
-        <v>4200</v>
+        <v>4403</v>
       </c>
       <c r="C20">
-        <v>5078.03</v>
+        <v>5751.26</v>
       </c>
       <c r="D20" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21">
-        <v>4403</v>
+        <v>4301</v>
       </c>
       <c r="B21">
-        <v>4101</v>
+        <v>4403</v>
       </c>
       <c r="C21">
-        <v>4898.55</v>
+        <v>5646.4</v>
       </c>
       <c r="D21" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22">
-        <v>2000</v>
+        <v>4403</v>
       </c>
       <c r="B22">
-        <v>4200</v>
+        <v>4203</v>
       </c>
       <c r="C22">
-        <v>4679.19</v>
+        <v>4808.26</v>
       </c>
       <c r="D22" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23">
+        <v>4108</v>
+      </c>
+      <c r="B23">
         <v>4104</v>
       </c>
-      <c r="B23">
-        <v>4304</v>
-      </c>
       <c r="C23">
-        <v>4390.42</v>
+        <v>4213.59</v>
       </c>
       <c r="D23" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -878,49 +875,49 @@
         <v>4100</v>
       </c>
       <c r="C24">
-        <v>4205.84</v>
+        <v>4061.11</v>
       </c>
       <c r="D24" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25">
-        <v>4400</v>
+        <v>4108</v>
       </c>
       <c r="B25">
-        <v>4403</v>
+        <v>4404</v>
       </c>
       <c r="C25">
-        <v>4125.72</v>
+        <v>4047.97</v>
       </c>
       <c r="D25" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26">
-        <v>4201</v>
+        <v>4304</v>
       </c>
       <c r="B26">
-        <v>4203</v>
+        <v>4301</v>
       </c>
       <c r="C26">
-        <v>3932.43</v>
+        <v>4035.02</v>
       </c>
       <c r="D26" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27">
-        <v>4203</v>
+        <v>4108</v>
       </c>
       <c r="B27">
-        <v>4302</v>
+        <v>4200</v>
       </c>
       <c r="C27">
-        <v>3876.68</v>
+        <v>3654.49</v>
       </c>
       <c r="D27" t="s">
         <v>24</v>
@@ -928,27 +925,27 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28">
-        <v>4403</v>
+        <v>4105</v>
       </c>
       <c r="B28">
-        <v>4108</v>
+        <v>4302</v>
       </c>
       <c r="C28">
-        <v>3631.78</v>
+        <v>3612.71</v>
       </c>
       <c r="D28" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29">
-        <v>4100</v>
+        <v>4301</v>
       </c>
       <c r="B29">
-        <v>4101</v>
+        <v>2000</v>
       </c>
       <c r="C29">
-        <v>3377.09</v>
+        <v>3523.27</v>
       </c>
       <c r="D29" t="s">
         <v>25</v>
@@ -956,86 +953,86 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30">
-        <v>4302</v>
+        <v>4201</v>
       </c>
       <c r="B30">
         <v>4200</v>
       </c>
       <c r="C30">
-        <v>3330.67</v>
+        <v>3388.73</v>
       </c>
       <c r="D30" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31">
-        <v>4200</v>
+        <v>4401</v>
       </c>
       <c r="B31">
-        <v>4302</v>
+        <v>4404</v>
       </c>
       <c r="C31">
-        <v>3226.3</v>
+        <v>3336.89</v>
       </c>
       <c r="D31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32">
-        <v>4108</v>
+        <v>4200</v>
       </c>
       <c r="B32">
-        <v>4404</v>
+        <v>4403</v>
       </c>
       <c r="C32">
-        <v>3058.57</v>
+        <v>3065.88</v>
       </c>
       <c r="D32" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33">
-        <v>4301</v>
+        <v>4101</v>
       </c>
       <c r="B33">
-        <v>4104</v>
+        <v>4100</v>
       </c>
       <c r="C33">
-        <v>2793.49</v>
+        <v>2948.67</v>
       </c>
       <c r="D33" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34">
-        <v>2000</v>
+        <v>4301</v>
       </c>
       <c r="B34">
-        <v>4304</v>
+        <v>4302</v>
       </c>
       <c r="C34">
-        <v>2521.22</v>
+        <v>2839.45</v>
       </c>
       <c r="D34" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35">
-        <v>4301</v>
+        <v>4203</v>
       </c>
       <c r="B35">
-        <v>2000</v>
+        <v>4200</v>
       </c>
       <c r="C35">
-        <v>2480.41</v>
+        <v>2808.28</v>
       </c>
       <c r="D35" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -1043,377 +1040,377 @@
         <v>4100</v>
       </c>
       <c r="B36">
-        <v>4304</v>
+        <v>4101</v>
       </c>
       <c r="C36">
-        <v>2413.47</v>
+        <v>2558.79</v>
       </c>
       <c r="D36" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37">
+        <v>4105</v>
+      </c>
+      <c r="B37">
         <v>4203</v>
       </c>
-      <c r="B37">
-        <v>4304</v>
-      </c>
       <c r="C37">
-        <v>2220.49</v>
+        <v>2414.28</v>
       </c>
       <c r="D37" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38">
-        <v>4108</v>
+        <v>4301</v>
       </c>
       <c r="B38">
-        <v>4203</v>
+        <v>4104</v>
       </c>
       <c r="C38">
-        <v>2088.84</v>
+        <v>2312.59</v>
       </c>
       <c r="D38" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39">
-        <v>4108</v>
+        <v>4100</v>
       </c>
       <c r="B39">
         <v>4104</v>
       </c>
       <c r="C39">
-        <v>2052.91</v>
+        <v>2244</v>
       </c>
       <c r="D39" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40">
-        <v>4400</v>
+        <v>4403</v>
       </c>
       <c r="B40">
-        <v>4304</v>
+        <v>4105</v>
       </c>
       <c r="C40">
-        <v>1924.31</v>
+        <v>2242.14</v>
       </c>
       <c r="D40" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41">
-        <v>4201</v>
+        <v>4104</v>
       </c>
       <c r="B41">
-        <v>4403</v>
+        <v>4108</v>
       </c>
       <c r="C41">
-        <v>1719.35</v>
+        <v>1915.22</v>
       </c>
       <c r="D41" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42">
-        <v>4108</v>
+        <v>4403</v>
       </c>
       <c r="B42">
-        <v>4105</v>
+        <v>4404</v>
       </c>
       <c r="C42">
-        <v>1693.85</v>
+        <v>1706.21</v>
       </c>
       <c r="D42" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43">
-        <v>4108</v>
+        <v>4104</v>
       </c>
       <c r="B43">
-        <v>4304</v>
+        <v>4302</v>
       </c>
       <c r="C43">
-        <v>1593.5</v>
+        <v>1640.03</v>
       </c>
       <c r="D43" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44">
-        <v>4400</v>
+        <v>4403</v>
       </c>
       <c r="B44">
-        <v>4203</v>
+        <v>4200</v>
       </c>
       <c r="C44">
-        <v>1502.9</v>
+        <v>1501.5</v>
       </c>
       <c r="D44" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45">
-        <v>4201</v>
+        <v>4200</v>
       </c>
       <c r="B45">
-        <v>4301</v>
+        <v>4401</v>
       </c>
       <c r="C45">
-        <v>1494.86</v>
+        <v>1483.27</v>
       </c>
       <c r="D45" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46">
-        <v>4400</v>
+        <v>4104</v>
       </c>
       <c r="B46">
-        <v>4404</v>
+        <v>4403</v>
       </c>
       <c r="C46">
-        <v>1429</v>
+        <v>1387.05</v>
       </c>
       <c r="D46" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47">
-        <v>4200</v>
+        <v>4201</v>
       </c>
       <c r="B47">
-        <v>4301</v>
+        <v>4404</v>
       </c>
       <c r="C47">
-        <v>1421.02</v>
+        <v>1198.21</v>
       </c>
       <c r="D47" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48">
-        <v>4201</v>
+        <v>4108</v>
       </c>
       <c r="B48">
-        <v>4401</v>
+        <v>4400</v>
       </c>
       <c r="C48">
-        <v>1402.72</v>
+        <v>1131.3</v>
       </c>
       <c r="D48" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49">
-        <v>4400</v>
+        <v>4203</v>
       </c>
       <c r="B49">
-        <v>4101</v>
+        <v>4403</v>
       </c>
       <c r="C49">
-        <v>1319.22</v>
+        <v>1114.05</v>
       </c>
       <c r="D49" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50">
-        <v>4301</v>
+        <v>4404</v>
       </c>
       <c r="B50">
-        <v>4101</v>
+        <v>4401</v>
       </c>
       <c r="C50">
-        <v>1297.48</v>
+        <v>1112.57</v>
       </c>
       <c r="D50" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51">
-        <v>4108</v>
+        <v>4100</v>
       </c>
       <c r="B51">
-        <v>4400</v>
+        <v>4401</v>
       </c>
       <c r="C51">
-        <v>1180.39</v>
+        <v>1106.18</v>
       </c>
       <c r="D51" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52">
-        <v>4203</v>
+        <v>4108</v>
       </c>
       <c r="B52">
-        <v>4105</v>
+        <v>2000</v>
       </c>
       <c r="C52">
-        <v>908.77</v>
+        <v>1068.66</v>
       </c>
       <c r="D52" t="s">
-        <v>40</v>
+        <v>8</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53">
-        <v>4200</v>
+        <v>4104</v>
       </c>
       <c r="B53">
-        <v>4101</v>
+        <v>2000</v>
       </c>
       <c r="C53">
-        <v>867.7</v>
+        <v>954.96</v>
       </c>
       <c r="D53" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54">
-        <v>4201</v>
+        <v>4403</v>
       </c>
       <c r="B54">
-        <v>4404</v>
+        <v>4302</v>
       </c>
       <c r="C54">
-        <v>801.23</v>
+        <v>928.78</v>
       </c>
       <c r="D54" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55">
-        <v>4401</v>
+        <v>4200</v>
       </c>
       <c r="B55">
-        <v>4404</v>
+        <v>4302</v>
       </c>
       <c r="C55">
-        <v>797.3099999999999</v>
+        <v>808.15</v>
       </c>
       <c r="D55" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="56" spans="1:4">
       <c r="A56">
-        <v>4105</v>
+        <v>4203</v>
       </c>
       <c r="B56">
-        <v>4403</v>
+        <v>4301</v>
       </c>
       <c r="C56">
-        <v>758.36</v>
+        <v>771.0700000000001</v>
       </c>
       <c r="D56" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57">
-        <v>4203</v>
+        <v>4301</v>
       </c>
       <c r="B57">
-        <v>4401</v>
+        <v>4201</v>
       </c>
       <c r="C57">
-        <v>603.6700000000001</v>
+        <v>638.46</v>
       </c>
       <c r="D57" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58">
-        <v>4203</v>
+        <v>4101</v>
       </c>
       <c r="B58">
-        <v>4301</v>
+        <v>4108</v>
       </c>
       <c r="C58">
-        <v>598.7</v>
+        <v>585.88</v>
       </c>
       <c r="D58" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59">
+        <v>4301</v>
+      </c>
+      <c r="B59">
         <v>4100</v>
       </c>
-      <c r="B59">
-        <v>4404</v>
-      </c>
       <c r="C59">
-        <v>553.9400000000001</v>
+        <v>585.53</v>
       </c>
       <c r="D59" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="60" spans="1:4">
       <c r="A60">
-        <v>4101</v>
+        <v>4200</v>
       </c>
       <c r="B60">
-        <v>4404</v>
+        <v>4400</v>
       </c>
       <c r="C60">
-        <v>547.55</v>
+        <v>565.89</v>
       </c>
       <c r="D60" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
     <row r="61" spans="1:4">
       <c r="A61">
-        <v>4200</v>
+        <v>4403</v>
       </c>
       <c r="B61">
-        <v>4404</v>
+        <v>4400</v>
       </c>
       <c r="C61">
-        <v>542.24</v>
+        <v>499.95</v>
       </c>
       <c r="D61" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="62" spans="1:4">
       <c r="A62">
-        <v>4304</v>
+        <v>4108</v>
       </c>
       <c r="B62">
-        <v>4301</v>
+        <v>4302</v>
       </c>
       <c r="C62">
-        <v>476.2</v>
+        <v>488.5</v>
       </c>
       <c r="D62" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -1424,259 +1421,259 @@
         <v>4304</v>
       </c>
       <c r="C63">
-        <v>447.26</v>
+        <v>482.18</v>
       </c>
       <c r="D63" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
     </row>
     <row r="64" spans="1:4">
       <c r="A64">
-        <v>4101</v>
+        <v>4304</v>
       </c>
       <c r="B64">
-        <v>4401</v>
+        <v>4104</v>
       </c>
       <c r="C64">
-        <v>403.57</v>
+        <v>468</v>
       </c>
       <c r="D64" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="65" spans="1:4">
       <c r="A65">
-        <v>4201</v>
+        <v>4302</v>
       </c>
       <c r="B65">
-        <v>4105</v>
+        <v>4403</v>
       </c>
       <c r="C65">
-        <v>300.07</v>
+        <v>463.82</v>
       </c>
       <c r="D65" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
     </row>
     <row r="66" spans="1:4">
       <c r="A66">
-        <v>4301</v>
+        <v>4302</v>
       </c>
       <c r="B66">
-        <v>4203</v>
+        <v>4304</v>
       </c>
       <c r="C66">
-        <v>251.69</v>
+        <v>389.03</v>
       </c>
       <c r="D66" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
     </row>
     <row r="67" spans="1:4">
       <c r="A67">
-        <v>4203</v>
+        <v>4108</v>
       </c>
       <c r="B67">
-        <v>4108</v>
+        <v>4105</v>
       </c>
       <c r="C67">
-        <v>226.94</v>
+        <v>273.76</v>
       </c>
       <c r="D67" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="68" spans="1:4">
       <c r="A68">
-        <v>4401</v>
+        <v>4302</v>
       </c>
       <c r="B68">
-        <v>4101</v>
+        <v>2000</v>
       </c>
       <c r="C68">
-        <v>199.27</v>
+        <v>271.19</v>
       </c>
       <c r="D68" t="s">
-        <v>17</v>
+        <v>49</v>
       </c>
     </row>
     <row r="69" spans="1:4">
       <c r="A69">
-        <v>4301</v>
+        <v>4304</v>
       </c>
       <c r="B69">
-        <v>4201</v>
+        <v>4403</v>
       </c>
       <c r="C69">
-        <v>159.37</v>
+        <v>245.63</v>
       </c>
       <c r="D69" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="70" spans="1:4">
       <c r="A70">
+        <v>4101</v>
+      </c>
+      <c r="B70">
         <v>4105</v>
       </c>
-      <c r="B70">
-        <v>4200</v>
-      </c>
       <c r="C70">
-        <v>136.09</v>
+        <v>231.28</v>
       </c>
       <c r="D70" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
     </row>
     <row r="71" spans="1:4">
       <c r="A71">
-        <v>4104</v>
+        <v>2000</v>
       </c>
       <c r="B71">
-        <v>4401</v>
+        <v>4304</v>
       </c>
       <c r="C71">
-        <v>109.05</v>
+        <v>180</v>
       </c>
       <c r="D71" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="72" spans="1:4">
       <c r="A72">
-        <v>4200</v>
+        <v>4104</v>
       </c>
       <c r="B72">
-        <v>4201</v>
+        <v>4401</v>
       </c>
       <c r="C72">
-        <v>108.37</v>
+        <v>175.27</v>
       </c>
       <c r="D72" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="73" spans="1:4">
       <c r="A73">
-        <v>4302</v>
+        <v>4400</v>
       </c>
       <c r="B73">
-        <v>4100</v>
+        <v>4101</v>
       </c>
       <c r="C73">
-        <v>93.33</v>
+        <v>168</v>
       </c>
       <c r="D73" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="74" spans="1:4">
       <c r="A74">
-        <v>4100</v>
+        <v>4101</v>
       </c>
       <c r="B74">
-        <v>4401</v>
+        <v>4404</v>
       </c>
       <c r="C74">
-        <v>84.48</v>
+        <v>139.81</v>
       </c>
       <c r="D74" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
     </row>
     <row r="75" spans="1:4">
       <c r="A75">
-        <v>4403</v>
+        <v>4101</v>
       </c>
       <c r="B75">
-        <v>4404</v>
+        <v>4104</v>
       </c>
       <c r="C75">
-        <v>72.62</v>
+        <v>129.75</v>
       </c>
       <c r="D75" t="s">
-        <v>55</v>
+        <v>36</v>
       </c>
     </row>
     <row r="76" spans="1:4">
       <c r="A76">
-        <v>4302</v>
+        <v>4304</v>
       </c>
       <c r="B76">
-        <v>4401</v>
+        <v>2000</v>
       </c>
       <c r="C76">
-        <v>47.35</v>
+        <v>113.95</v>
       </c>
       <c r="D76" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="77" spans="1:4">
       <c r="A77">
-        <v>4302</v>
+        <v>4203</v>
       </c>
       <c r="B77">
-        <v>4108</v>
+        <v>4101</v>
       </c>
       <c r="C77">
-        <v>40.9</v>
+        <v>88.67</v>
       </c>
       <c r="D77" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="78" spans="1:4">
       <c r="A78">
-        <v>4302</v>
+        <v>4301</v>
       </c>
       <c r="B78">
-        <v>4104</v>
+        <v>4203</v>
       </c>
       <c r="C78">
-        <v>14.4</v>
+        <v>87.96000000000001</v>
       </c>
       <c r="D78" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="79" spans="1:4">
       <c r="A79">
-        <v>4403</v>
+        <v>4104</v>
       </c>
       <c r="B79">
-        <v>4401</v>
+        <v>4200</v>
       </c>
       <c r="C79">
-        <v>13.39</v>
+        <v>73.67</v>
       </c>
       <c r="D79" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
     </row>
     <row r="80" spans="1:4">
       <c r="A80">
-        <v>4105</v>
+        <v>4203</v>
       </c>
       <c r="B80">
-        <v>4404</v>
+        <v>4201</v>
       </c>
       <c r="C80">
-        <v>11.81</v>
+        <v>70.27</v>
       </c>
       <c r="D80" t="s">
-        <v>56</v>
+        <v>36</v>
       </c>
     </row>
     <row r="81" spans="1:4">
       <c r="A81">
-        <v>4403</v>
+        <v>4104</v>
       </c>
       <c r="B81">
-        <v>4400</v>
+        <v>4304</v>
       </c>
       <c r="C81">
-        <v>9.640000000000001</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="D81" t="s">
         <v>52</v>
@@ -1684,58 +1681,100 @@
     </row>
     <row r="82" spans="1:4">
       <c r="A82">
-        <v>4301</v>
+        <v>4400</v>
       </c>
       <c r="B82">
-        <v>4404</v>
+        <v>4200</v>
       </c>
       <c r="C82">
-        <v>7.2</v>
+        <v>62.1</v>
       </c>
       <c r="D82" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
     </row>
     <row r="83" spans="1:4">
       <c r="A83">
-        <v>4301</v>
+        <v>4203</v>
       </c>
       <c r="B83">
-        <v>4200</v>
+        <v>4304</v>
       </c>
       <c r="C83">
-        <v>3.07</v>
+        <v>60.54</v>
       </c>
       <c r="D83" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="84" spans="1:4">
       <c r="A84">
-        <v>4404</v>
+        <v>4200</v>
       </c>
       <c r="B84">
-        <v>4401</v>
+        <v>4201</v>
       </c>
       <c r="C84">
-        <v>1.73</v>
+        <v>44.68000000000001</v>
       </c>
       <c r="D84" t="s">
-        <v>38</v>
+        <v>55</v>
       </c>
     </row>
     <row r="85" spans="1:4">
       <c r="A85">
-        <v>4203</v>
+        <v>4105</v>
       </c>
       <c r="B85">
-        <v>4201</v>
+        <v>4101</v>
       </c>
       <c r="C85">
-        <v>1.72</v>
+        <v>35.11</v>
       </c>
       <c r="D85" t="s">
-        <v>50</v>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4">
+      <c r="A86">
+        <v>4304</v>
+      </c>
+      <c r="B86">
+        <v>4302</v>
+      </c>
+      <c r="C86">
+        <v>34.36</v>
+      </c>
+      <c r="D86" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4">
+      <c r="A87">
+        <v>4104</v>
+      </c>
+      <c r="B87">
+        <v>4100</v>
+      </c>
+      <c r="C87">
+        <v>24.1</v>
+      </c>
+      <c r="D87" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4">
+      <c r="A88">
+        <v>4400</v>
+      </c>
+      <c r="B88">
+        <v>4403</v>
+      </c>
+      <c r="C88">
+        <v>4.97</v>
+      </c>
+      <c r="D88" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>